<commit_message>
End of The Project
</commit_message>
<xml_diff>
--- a/notes/Anxiety-Model-Versus.xlsx
+++ b/notes/Anxiety-Model-Versus.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Visual Studio Code\Anxiety-Analysis-ML\notes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A98C379-7795-467F-B6CC-43D27773881A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9924E650-54A5-404C-A130-87241D210D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="110">
   <si>
     <t>Logistic Regression</t>
   </si>
@@ -315,34 +315,46 @@
     <t>anxiety_model_20250510_2039</t>
   </si>
   <si>
-    <t>→Anksiyete (98.64%)</t>
-  </si>
-  <si>
-    <t>→Anksiyete (59.12%)</t>
-  </si>
-  <si>
-    <t>→Anksiyete (98.38%)</t>
-  </si>
-  <si>
-    <t>→Normal (18.99%)</t>
-  </si>
-  <si>
-    <t>→Anksiyete (87.41%)</t>
-  </si>
-  <si>
-    <t>→Anksiyete (83.68%)</t>
-  </si>
-  <si>
-    <t>→Anksiyete (94.38%)</t>
-  </si>
-  <si>
-    <t>→Anksiyete (64.69%)</t>
-  </si>
-  <si>
-    <t>→Anksiyete (96.03%)</t>
-  </si>
-  <si>
-    <t>→Normal (47.84%)</t>
+    <t>Anksiyete (98.64%)</t>
+  </si>
+  <si>
+    <t>Anksiyete (59.12%)</t>
+  </si>
+  <si>
+    <t>Anksiyete (98.38%)</t>
+  </si>
+  <si>
+    <t>Normal (18.99%)</t>
+  </si>
+  <si>
+    <t>Anksiyete (87.41%)</t>
+  </si>
+  <si>
+    <t>Anksiyete (83.68%)</t>
+  </si>
+  <si>
+    <t>Anksiyete (94.38%)</t>
+  </si>
+  <si>
+    <t>Anksiyete (64.69%)</t>
+  </si>
+  <si>
+    <t>Anksiyete (96.03%)</t>
+  </si>
+  <si>
+    <t>Normal (47.84%)</t>
+  </si>
+  <si>
+    <t>:CROSS VALIDATION  ACCURACY</t>
+  </si>
+  <si>
+    <t>:ACCURACY</t>
+  </si>
+  <si>
+    <t>:F1 SCORE</t>
+  </si>
+  <si>
+    <t>:ROC AUC SCORE</t>
   </si>
 </sst>
 </file>
@@ -458,7 +470,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
@@ -488,6 +500,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -778,8 +793,10 @@
   <dimension ref="A1:H27"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="33.44140625" customWidth="1"/>
-    <col min="2" max="8" width="44.33203125" customWidth="1"/>
+    <col min="1" max="1" width="36.6640625" customWidth="1"/>
+    <col min="2" max="6" width="44.33203125" customWidth="1"/>
+    <col min="7" max="7" width="33.6640625" customWidth="1"/>
+    <col min="8" max="8" width="44.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="18" x14ac:dyDescent="0.3">
@@ -1275,7 +1292,9 @@
       <c r="F24" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="G24" s="10"/>
+      <c r="G24" s="11" t="s">
+        <v>106</v>
+      </c>
       <c r="H24" s="10"/>
     </row>
     <row r="25" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
@@ -1297,7 +1316,9 @@
       <c r="F25" s="10" t="s">
         <v>92</v>
       </c>
-      <c r="G25" s="10"/>
+      <c r="G25" s="11" t="s">
+        <v>107</v>
+      </c>
       <c r="H25" s="10"/>
     </row>
     <row r="26" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
@@ -1319,7 +1340,9 @@
       <c r="F26" s="10" t="s">
         <v>93</v>
       </c>
-      <c r="G26" s="10"/>
+      <c r="G26" s="11" t="s">
+        <v>108</v>
+      </c>
       <c r="H26" s="10"/>
     </row>
     <row r="27" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
@@ -1341,7 +1364,9 @@
       <c r="F27" s="10" t="s">
         <v>94</v>
       </c>
-      <c r="G27" s="10"/>
+      <c r="G27" s="11" t="s">
+        <v>109</v>
+      </c>
       <c r="H27" s="10"/>
     </row>
   </sheetData>

</xml_diff>